<commit_message>
Republish Augsburg_2025_WC: Kayak Cross individual (Time Trials) RANK from official classification (94 cells; maintainer 2026-10-21)
</commit_message>
<xml_diff>
--- a/events/Augsburg_2025_WC/Augsburg_2025_WC_start.xlsx
+++ b/events/Augsburg_2025_WC/Augsburg_2025_WC_start.xlsx
@@ -22989,6 +22989,11 @@
       <c r="K380" t="n">
         <v>379</v>
       </c>
+      <c r="M380" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="R380" t="inlineStr">
         <is>
           <t>LUKNAROVA Emanuela</t>
@@ -23052,6 +23057,11 @@
       <c r="K381" t="n">
         <v>380</v>
       </c>
+      <c r="M381" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
       <c r="R381" t="inlineStr">
         <is>
           <t>HORLOVA Valentyna</t>
@@ -23115,6 +23125,11 @@
       <c r="K382" t="n">
         <v>381</v>
       </c>
+      <c r="M382" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="R382" t="inlineStr">
         <is>
           <t>NAGASU Momoka</t>
@@ -23178,6 +23193,11 @@
       <c r="K383" t="n">
         <v>382</v>
       </c>
+      <c r="M383" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="R383" t="inlineStr">
         <is>
           <t>PITCHER FARRELL Cleo</t>
@@ -23241,6 +23261,11 @@
       <c r="K384" t="n">
         <v>383</v>
       </c>
+      <c r="M384" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="R384" t="inlineStr">
         <is>
           <t>HORLOVA Oleksandra</t>
@@ -23367,6 +23392,11 @@
       <c r="K386" t="n">
         <v>385</v>
       </c>
+      <c r="M386" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="R386" t="inlineStr">
         <is>
           <t>PELLICER CHICA Laura</t>
@@ -23430,6 +23460,11 @@
       <c r="K387" t="n">
         <v>386</v>
       </c>
+      <c r="M387" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="R387" t="inlineStr">
         <is>
           <t>CROSBEE Sarah</t>
@@ -23493,6 +23528,11 @@
       <c r="K388" t="n">
         <v>387</v>
       </c>
+      <c r="M388" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="R388" t="inlineStr">
         <is>
           <t>REX Rosie</t>
@@ -23619,6 +23659,11 @@
       <c r="K390" t="n">
         <v>389</v>
       </c>
+      <c r="M390" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="R390" t="inlineStr">
         <is>
           <t>ARREGUI Olatz</t>
@@ -23682,6 +23727,11 @@
       <c r="K391" t="n">
         <v>390</v>
       </c>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="R391" t="inlineStr">
         <is>
           <t>O'CALLAGHAN Georgia</t>
@@ -23745,6 +23795,11 @@
       <c r="K392" t="n">
         <v>391</v>
       </c>
+      <c r="M392" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="R392" t="inlineStr">
         <is>
           <t>ALTMAN Marcella</t>
@@ -23808,6 +23863,11 @@
       <c r="K393" t="n">
         <v>392</v>
       </c>
+      <c r="M393" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
       <c r="R393" t="inlineStr">
         <is>
           <t>HERZOG Andrea</t>
@@ -23871,6 +23931,11 @@
       <c r="K394" t="n">
         <v>393</v>
       </c>
+      <c r="M394" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="R394" t="inlineStr">
         <is>
           <t>SAMKOVA Olga</t>
@@ -23934,6 +23999,11 @@
       <c r="K395" t="n">
         <v>394</v>
       </c>
+      <c r="M395" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="R395" t="inlineStr">
         <is>
           <t>STANOVSKA Sona</t>
@@ -23997,6 +24067,11 @@
       <c r="K396" t="n">
         <v>395</v>
       </c>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="R396" t="inlineStr">
         <is>
           <t>LEAVER Lois</t>
@@ -24060,6 +24135,11 @@
       <c r="K397" t="n">
         <v>396</v>
       </c>
+      <c r="M397" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="R397" t="inlineStr">
         <is>
           <t>LI Shiting</t>
@@ -24123,6 +24203,11 @@
       <c r="K398" t="n">
         <v>397</v>
       </c>
+      <c r="M398" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="R398" t="inlineStr">
         <is>
           <t>BAYN Nele</t>
@@ -24186,6 +24271,11 @@
       <c r="K399" t="n">
         <v>398</v>
       </c>
+      <c r="M399" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="R399" t="inlineStr">
         <is>
           <t>PINTERIC Naja</t>
@@ -24249,6 +24339,11 @@
       <c r="K400" t="n">
         <v>399</v>
       </c>
+      <c r="M400" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="R400" t="inlineStr">
         <is>
           <t>NOVAK Ajda</t>
@@ -24312,6 +24407,11 @@
       <c r="K401" t="n">
         <v>400</v>
       </c>
+      <c r="M401" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="R401" t="inlineStr">
         <is>
           <t>TEUNISSEN Lena</t>
@@ -24375,6 +24475,11 @@
       <c r="K402" t="n">
         <v>401</v>
       </c>
+      <c r="M402" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
       <c r="R402" t="inlineStr">
         <is>
           <t>HOCEVAR Eva Alina</t>
@@ -24438,6 +24543,11 @@
       <c r="K403" t="n">
         <v>402</v>
       </c>
+      <c r="M403" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="R403" t="inlineStr">
         <is>
           <t>US Viktoriia</t>
@@ -24501,6 +24611,11 @@
       <c r="K404" t="n">
         <v>403</v>
       </c>
+      <c r="M404" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="R404" t="inlineStr">
         <is>
           <t>SABATTINI Chiara</t>
@@ -24564,6 +24679,11 @@
       <c r="K405" t="n">
         <v>404</v>
       </c>
+      <c r="M405" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="R405" t="inlineStr">
         <is>
           <t>BEKOVA Katerina</t>
@@ -24627,6 +24747,11 @@
       <c r="K406" t="n">
         <v>405</v>
       </c>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="R406" t="inlineStr">
         <is>
           <t>LAZKANO Miren</t>
@@ -24690,6 +24815,11 @@
       <c r="K407" t="n">
         <v>406</v>
       </c>
+      <c r="M407" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="R407" t="inlineStr">
         <is>
           <t>SATILA Ana</t>
@@ -24753,6 +24883,11 @@
       <c r="K408" t="n">
         <v>407</v>
       </c>
+      <c r="M408" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="R408" t="inlineStr">
         <is>
           <t>DORIA Monica</t>
@@ -24816,6 +24951,11 @@
       <c r="K409" t="n">
         <v>408</v>
       </c>
+      <c r="M409" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="R409" t="inlineStr">
         <is>
           <t>ESTACIA NETA Omira</t>
@@ -24879,6 +25019,11 @@
       <c r="K410" t="n">
         <v>409</v>
       </c>
+      <c r="M410" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="R410" t="inlineStr">
         <is>
           <t>KNEBLOVA Tereza</t>
@@ -24942,6 +25087,11 @@
       <c r="K411" t="n">
         <v>410</v>
       </c>
+      <c r="M411" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="R411" t="inlineStr">
         <is>
           <t>SETCHELL Nikita</t>
@@ -25005,6 +25155,11 @@
       <c r="K412" t="n">
         <v>411</v>
       </c>
+      <c r="M412" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="R412" t="inlineStr">
         <is>
           <t>VUITTON Emma</t>
@@ -25068,6 +25223,11 @@
       <c r="K413" t="n">
         <v>412</v>
       </c>
+      <c r="M413" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="R413" t="inlineStr">
         <is>
           <t>LEIBFARTH Evy</t>
@@ -25131,6 +25291,11 @@
       <c r="K414" t="n">
         <v>413</v>
       </c>
+      <c r="M414" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R414" t="inlineStr">
         <is>
           <t>FUNK Ricarda</t>
@@ -25194,6 +25359,11 @@
       <c r="K415" t="n">
         <v>414</v>
       </c>
+      <c r="M415" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="R415" t="inlineStr">
         <is>
           <t>MARX Alena</t>
@@ -25257,6 +25427,11 @@
       <c r="K416" t="n">
         <v>415</v>
       </c>
+      <c r="M416" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="R416" t="inlineStr">
         <is>
           <t>CHOURRAUT Maialen</t>
@@ -25320,6 +25495,11 @@
       <c r="K417" t="n">
         <v>416</v>
       </c>
+      <c r="M417" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="R417" t="inlineStr">
         <is>
           <t>FOX Noemie</t>
@@ -25383,6 +25563,11 @@
       <c r="K418" t="n">
         <v>417</v>
       </c>
+      <c r="M418" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="R418" t="inlineStr">
         <is>
           <t>PRIGENT Camille</t>
@@ -25446,6 +25631,11 @@
       <c r="K419" t="n">
         <v>418</v>
       </c>
+      <c r="M419" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="R419" t="inlineStr">
         <is>
           <t>HUG Angele</t>
@@ -25509,6 +25699,11 @@
       <c r="K420" t="n">
         <v>419</v>
       </c>
+      <c r="M420" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="R420" t="inlineStr">
         <is>
           <t>WOODS Kimberley</t>
@@ -25572,6 +25767,11 @@
       <c r="K421" t="n">
         <v>420</v>
       </c>
+      <c r="M421" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
       <c r="R421" t="inlineStr">
         <is>
           <t>RAHKOLA Visa</t>
@@ -25635,6 +25835,11 @@
       <c r="K422" t="n">
         <v>421</v>
       </c>
+      <c r="M422" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
       <c r="R422" t="inlineStr">
         <is>
           <t>LOOS Soren</t>
@@ -25698,6 +25903,11 @@
       <c r="K423" t="n">
         <v>422</v>
       </c>
+      <c r="M423" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="R423" t="inlineStr">
         <is>
           <t>KITAMURA Koki</t>
@@ -25761,6 +25971,11 @@
       <c r="K424" t="n">
         <v>423</v>
       </c>
+      <c r="M424" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
       <c r="R424" t="inlineStr">
         <is>
           <t>TARKKA Teijo</t>
@@ -25824,6 +26039,11 @@
       <c r="K425" t="n">
         <v>424</v>
       </c>
+      <c r="M425" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
       <c r="R425" t="inlineStr">
         <is>
           <t>NESHIME Daisuke</t>
@@ -25887,6 +26107,11 @@
       <c r="K426" t="n">
         <v>425</v>
       </c>
+      <c r="M426" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="R426" t="inlineStr">
         <is>
           <t>MISHIMA Yu</t>
@@ -25950,6 +26175,11 @@
       <c r="K427" t="n">
         <v>426</v>
       </c>
+      <c r="M427" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="R427" t="inlineStr">
         <is>
           <t>SKUBIK David</t>
@@ -26013,6 +26243,11 @@
       <c r="K428" t="n">
         <v>427</v>
       </c>
+      <c r="M428" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
       <c r="R428" t="inlineStr">
         <is>
           <t>MARIEN Martin</t>
@@ -26076,6 +26311,11 @@
       <c r="K429" t="n">
         <v>428</v>
       </c>
+      <c r="M429" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
       <c r="R429" t="inlineStr">
         <is>
           <t>CELMINS Ritvars</t>
@@ -26139,6 +26379,11 @@
       <c r="K430" t="n">
         <v>429</v>
       </c>
+      <c r="M430" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="R430" t="inlineStr">
         <is>
           <t>KRACHKO Arkhyp</t>
@@ -26202,6 +26447,11 @@
       <c r="K431" t="n">
         <v>430</v>
       </c>
+      <c r="M431" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
       <c r="R431" t="inlineStr">
         <is>
           <t>BARAT Andy</t>
@@ -26265,6 +26515,11 @@
       <c r="K432" t="n">
         <v>431</v>
       </c>
+      <c r="M432" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
       <c r="R432" t="inlineStr">
         <is>
           <t>DA SILVA Kaua</t>
@@ -26328,6 +26583,11 @@
       <c r="K433" t="n">
         <v>432</v>
       </c>
+      <c r="M433" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
       <c r="R433" t="inlineStr">
         <is>
           <t>ANDERSON Finn</t>
@@ -26454,6 +26714,11 @@
       <c r="K435" t="n">
         <v>434</v>
       </c>
+      <c r="M435" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
       <c r="R435" t="inlineStr">
         <is>
           <t>BOYD Trevor</t>
@@ -26580,6 +26845,11 @@
       <c r="K437" t="n">
         <v>436</v>
       </c>
+      <c r="M437" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="R437" t="inlineStr">
         <is>
           <t>LOCNIKAR Jan</t>
@@ -26643,6 +26913,11 @@
       <c r="K438" t="n">
         <v>437</v>
       </c>
+      <c r="M438" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
       <c r="R438" t="inlineStr">
         <is>
           <t>SOVKO Serhii</t>
@@ -26706,6 +26981,11 @@
       <c r="K439" t="n">
         <v>438</v>
       </c>
+      <c r="M439" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="R439" t="inlineStr">
         <is>
           <t>FRIEDENSON Kaelin</t>
@@ -26769,6 +27049,11 @@
       <c r="K440" t="n">
         <v>439</v>
       </c>
+      <c r="M440" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="R440" t="inlineStr">
         <is>
           <t>KREMSLEHNER Moritz</t>
@@ -26832,6 +27117,11 @@
       <c r="K441" t="n">
         <v>440</v>
       </c>
+      <c r="M441" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="R441" t="inlineStr">
         <is>
           <t>RUDORFER Martin</t>
@@ -26895,6 +27185,11 @@
       <c r="K442" t="n">
         <v>441</v>
       </c>
+      <c r="M442" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="R442" t="inlineStr">
         <is>
           <t>AUBERTIN Maxime</t>
@@ -26958,6 +27253,11 @@
       <c r="K443" t="n">
         <v>442</v>
       </c>
+      <c r="M443" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
       <c r="R443" t="inlineStr">
         <is>
           <t>FERRAZZI Xabier</t>
@@ -27021,6 +27321,11 @@
       <c r="K444" t="n">
         <v>443</v>
       </c>
+      <c r="M444" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="R444" t="inlineStr">
         <is>
           <t>LEITNER Mario</t>
@@ -27084,6 +27389,11 @@
       <c r="K445" t="n">
         <v>444</v>
       </c>
+      <c r="M445" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="R445" t="inlineStr">
         <is>
           <t>GRIGAR Jakub</t>
@@ -27147,6 +27457,11 @@
       <c r="K446" t="n">
         <v>445</v>
       </c>
+      <c r="M446" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
       <c r="R446" t="inlineStr">
         <is>
           <t>MCCREERY Alistair</t>
@@ -27273,6 +27588,11 @@
       <c r="K448" t="n">
         <v>447</v>
       </c>
+      <c r="M448" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
       <c r="R448" t="inlineStr">
         <is>
           <t>HALCIN Martin</t>
@@ -27336,6 +27656,11 @@
       <c r="K449" t="n">
         <v>448</v>
       </c>
+      <c r="M449" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="R449" t="inlineStr">
         <is>
           <t>OHRSTROM Isak</t>
@@ -27399,6 +27724,11 @@
       <c r="K450" t="n">
         <v>449</v>
       </c>
+      <c r="M450" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="R450" t="inlineStr">
         <is>
           <t>CURTIN Dominic</t>
@@ -27525,6 +27855,11 @@
       <c r="K452" t="n">
         <v>451</v>
       </c>
+      <c r="M452" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="R452" t="inlineStr">
         <is>
           <t>IVCHENKO Artem</t>
@@ -27588,6 +27923,11 @@
       <c r="K453" t="n">
         <v>452</v>
       </c>
+      <c r="M453" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="R453" t="inlineStr">
         <is>
           <t>SAVLI Jakob</t>
@@ -27651,6 +27991,11 @@
       <c r="K454" t="n">
         <v>453</v>
       </c>
+      <c r="M454" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="R454" t="inlineStr">
         <is>
           <t>COLLIER Nicholas</t>
@@ -27777,6 +28122,11 @@
       <c r="K456" t="n">
         <v>455</v>
       </c>
+      <c r="M456" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="R456" t="inlineStr">
         <is>
           <t>LONG Kyler James</t>
@@ -27840,6 +28190,11 @@
       <c r="K457" t="n">
         <v>456</v>
       </c>
+      <c r="M457" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
       <c r="R457" t="inlineStr">
         <is>
           <t>CASTRYCK Titouan</t>
@@ -27903,6 +28258,11 @@
       <c r="K458" t="n">
         <v>457</v>
       </c>
+      <c r="M458" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="R458" t="inlineStr">
         <is>
           <t>ROELLER Tillmann</t>
@@ -27966,6 +28326,11 @@
       <c r="K459" t="n">
         <v>458</v>
       </c>
+      <c r="M459" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="R459" t="inlineStr">
         <is>
           <t>NOVAK Matyas</t>
@@ -28029,6 +28394,11 @@
       <c r="K460" t="n">
         <v>459</v>
       </c>
+      <c r="M460" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="R460" t="inlineStr">
         <is>
           <t>HENGST Stefan</t>
@@ -28092,6 +28462,11 @@
       <c r="K461" t="n">
         <v>460</v>
       </c>
+      <c r="M461" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="R461" t="inlineStr">
         <is>
           <t>BALDONI Alex</t>
@@ -28155,6 +28530,11 @@
       <c r="K462" t="n">
         <v>461</v>
       </c>
+      <c r="M462" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="R462" t="inlineStr">
         <is>
           <t>LONG Merle</t>
@@ -28218,6 +28598,11 @@
       <c r="K463" t="n">
         <v>462</v>
       </c>
+      <c r="M463" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
       <c r="R463" t="inlineStr">
         <is>
           <t>KREJCI Jakub</t>
@@ -28281,6 +28666,11 @@
       <c r="K464" t="n">
         <v>463</v>
       </c>
+      <c r="M464" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
       <c r="R464" t="inlineStr">
         <is>
           <t>CHIARELLO Gelindo</t>
@@ -28344,6 +28734,11 @@
       <c r="K465" t="n">
         <v>464</v>
       </c>
+      <c r="M465" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="R465" t="inlineStr">
         <is>
           <t>DE COSTER Gabriel</t>
@@ -28407,6 +28802,11 @@
       <c r="K466" t="n">
         <v>465</v>
       </c>
+      <c r="M466" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="R466" t="inlineStr">
         <is>
           <t>DELFOUR Lucien</t>
@@ -28470,6 +28870,11 @@
       <c r="K467" t="n">
         <v>466</v>
       </c>
+      <c r="M467" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="R467" t="inlineStr">
         <is>
           <t>HOCEVAR Ziga Lin</t>
@@ -28533,6 +28938,11 @@
       <c r="K468" t="n">
         <v>467</v>
       </c>
+      <c r="M468" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="R468" t="inlineStr">
         <is>
           <t>QUAN Xin</t>
@@ -28596,6 +29006,11 @@
       <c r="K469" t="n">
         <v>468</v>
       </c>
+      <c r="M469" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R469" t="inlineStr">
         <is>
           <t>LEAVER Sam</t>
@@ -28659,6 +29074,11 @@
       <c r="K470" t="n">
         <v>469</v>
       </c>
+      <c r="M470" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="R470" t="inlineStr">
         <is>
           <t>OSCHMAUTZ Felix</t>
@@ -28722,6 +29142,11 @@
       <c r="K471" t="n">
         <v>470</v>
       </c>
+      <c r="M471" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="R471" t="inlineStr">
         <is>
           <t>ROHRER Jan</t>
@@ -28848,6 +29273,11 @@
       <c r="K473" t="n">
         <v>472</v>
       </c>
+      <c r="M473" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="R473" t="inlineStr">
         <is>
           <t>MADORE Mathurin</t>
@@ -28911,6 +29341,11 @@
       <c r="K474" t="n">
         <v>473</v>
       </c>
+      <c r="M474" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
       <c r="R474" t="inlineStr">
         <is>
           <t>GONCALVES Pedro</t>
@@ -28974,6 +29409,11 @@
       <c r="K475" t="n">
         <v>474</v>
       </c>
+      <c r="M475" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
       <c r="R475" t="inlineStr">
         <is>
           <t>HEGGE Noah</t>
@@ -29037,6 +29477,11 @@
       <c r="K476" t="n">
         <v>475</v>
       </c>
+      <c r="M476" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="R476" t="inlineStr">
         <is>
           <t>DICKSON Jonny</t>
@@ -29100,6 +29545,11 @@
       <c r="K477" t="n">
         <v>476</v>
       </c>
+      <c r="M477" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="R477" t="inlineStr">
         <is>
           <t>RENIA Benjamin</t>
@@ -29163,6 +29613,11 @@
       <c r="K478" t="n">
         <v>477</v>
       </c>
+      <c r="M478" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="R478" t="inlineStr">
         <is>
           <t>OCHOA Manuel</t>
@@ -29226,6 +29681,11 @@
       <c r="K479" t="n">
         <v>478</v>
       </c>
+      <c r="M479" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="R479" t="inlineStr">
         <is>
           <t>LLORENTE David</t>
@@ -29289,6 +29749,11 @@
       <c r="K480" t="n">
         <v>479</v>
       </c>
+      <c r="M480" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="R480" t="inlineStr">
         <is>
           <t>DOUGOUD Martin</t>
@@ -29351,6 +29816,11 @@
       </c>
       <c r="K481" t="n">
         <v>480</v>
+      </c>
+      <c r="M481" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="R481" t="inlineStr">
         <is>

</xml_diff>